<commit_message>
feat(qa): expand Mega Menu test cases to 28 TCs covering all sections, promo cards, tablet, and sticky header
</commit_message>
<xml_diff>
--- a/Sprint-3/MASTER_BACKUP_SPRINT_3/09_Mega_Menu/Mega_Menu_Test_Cases.xlsx
+++ b/Sprint-3/MASTER_BACKUP_SPRINT_3/09_Mega_Menu/Mega_Menu_Test_Cases.xlsx
@@ -397,16 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I29"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
     <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="55.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="55.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="65.83203125" customWidth="1"/>
+    <col min="6" max="6" width="55.83203125" customWidth="1"/>
+    <col min="7" max="7" width="60.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -453,9 +453,9 @@
         <v>User is on US staging homepage on desktop browser</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the homepage on desktop browser.
-2. Look at the top navigation menu.
-3. Verify all 9 main categories are visible: Indoor, Outdoor, Homewares, In Stock, Customisation, Projects, Inspiration, Support, Contact.</v>
+        <v xml:space="preserve">Step 1: Open the homepage on desktop browser.
+Step 2: Look at the top navigation menu.
+Step 3: Verify all 9 main categories are visible: Indoor, Outdoor, Homewares, In Stock, Customisation, Projects, Inspiration, Support, Contact.</v>
       </c>
       <c r="F2" t="str">
         <v>All 9 categories should be displayed in the correct order with proper spacing.</v>
@@ -484,9 +484,9 @@
         <v>User is on homepage on desktop</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "Indoor" in the main menu.
-2. Check the dropdown layout showing Furniture, Rugs, and Lighting columns.
-3. Click on a few subcategories like Sofas, Dining Tables, and Lounge Chairs to check navigation.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "Indoor" in the main menu.
+Step 2: Check the dropdown layout showing Furniture, Rugs, and Lighting columns.
+Step 3: Click on a few subcategories like Sofas, Dining Tables, and Lounge Chairs to check navigation.</v>
       </c>
       <c r="F3" t="str">
         <v>Dropdown should open smoothly, showing all columns and subcategory links clearly.</v>
@@ -515,9 +515,9 @@
         <v>Indoor dropdown menu is open</v>
       </c>
       <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover over "Indoor" to open the menu.
-2. Locate the "Outlet" link under Indoor.
-3. Click on the Outlet link or inspect its URL destination.</v>
+        <v xml:space="preserve">Step 1: Hover over "Indoor" to open the menu.
+Step 2: Locate the "Outlet" link under Indoor.
+Step 3: Click on the Outlet link or inspect its URL destination.</v>
       </c>
       <c r="F4" t="str">
         <v>The link should navigate to the US outlet page on mcstaging2.globewest.com.</v>
@@ -546,9 +546,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "Outdoor" in the main menu.
-2. Check columns and subcategory links (Tables, Chairs, Sofas, Accessories).
-3. Check the destination URL for the Outdoor Outlet link.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "Outdoor" in the main menu.
+Step 2: Check columns and subcategory links (Tables, Chairs, Sofas, Accessories).
+Step 3: Check the destination URL for the Outdoor Outlet link.</v>
       </c>
       <c r="F5" t="str">
         <v>All links should stay on the US store without redirecting to Australian domain.</v>
@@ -577,9 +577,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "Homewares" in the main menu.
-2. Check the subcategory links under Homewares.
-3. Check the destination URL for the Homewares Outlet link.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "Homewares" in the main menu.
+Step 2: Check the subcategory links under Homewares.
+Step 3: Check the destination URL for the Homewares Outlet link.</v>
       </c>
       <c r="F6" t="str">
         <v>All links should point to the US store.</v>
@@ -608,9 +608,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "In Stock" in the main navigation.
-2. Check all category group links (In Stock Indoor, In Stock Outdoor, etc.).
-3. Click on "In Stock Indoor" to test navigation.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "In Stock" in the main navigation.
+Step 2: Check all category group links (In Stock Indoor, In Stock Outdoor, etc.).
+Step 3: Click on "In Stock Indoor" to test navigation.</v>
       </c>
       <c r="F7" t="str">
         <v>Menu should open cleanly and links should direct to US in-stock product listings.</v>
@@ -639,9 +639,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover over "Customisation" and click the link.
-2. Hover over "Projects" and click a project gallery link.
-3. Confirm that both pages load properly.</v>
+        <v xml:space="preserve">Step 1: Hover over "Customisation" and click the link.
+Step 2: Hover over "Projects" and click a project gallery link.
+Step 3: Confirm that both pages load properly.</v>
       </c>
       <c r="F8" t="str">
         <v>Both links should load their respective US pages without any errors.</v>
@@ -670,9 +670,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "Inspiration".
-2. Review lookbooks and design inspiration links.
-3. Click on a lookbook link to test navigation.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "Inspiration".
+Step 2: Review lookbooks and design inspiration links.
+Step 3: Click on a lookbook link to test navigation.</v>
       </c>
       <c r="F9" t="str">
         <v>All links should navigate to US blog and lookbook pages.</v>
@@ -701,9 +701,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "Support" in header.
-2. Review all links under Support (Help Centre, Care, Warranty, Outlet).
-3. Check destination URLs for all links.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "Support" in header.
+Step 2: Review all links under Support (Help Centre, Care, Warranty, Outlet).
+Step 3: Check destination URLs for all links.</v>
       </c>
       <c r="F10" t="str">
         <v>All support links should open US customer care and FAQ pages.</v>
@@ -732,9 +732,9 @@
         <v>User on desktop view</v>
       </c>
       <c r="E11" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover over or click "Contact" in header menu.
-2. Click on "Contact Us" or "Book a Showroom".
-3. Verify page navigation.</v>
+        <v xml:space="preserve">Step 1: Hover over or click "Contact" in header menu.
+Step 2: Click on "Contact Us" or "Book a Showroom".
+Step 3: Verify page navigation.</v>
       </c>
       <c r="F11" t="str">
         <v>User should be taken to the US contact and showroom booking page.</v>
@@ -763,10 +763,10 @@
         <v>Mobile view (390x844 on mobile device)</v>
       </c>
       <c r="E12" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website on mobile browser.
-2. Tap the hamburger menu icon (three lines) in the header.
-3. Verify that the side menu slides open smoothly.
-4. Check that all 9 categories are listed.</v>
+        <v xml:space="preserve">Step 1: Open the website on mobile browser.
+Step 2: Tap the hamburger menu icon (three lines) in the header.
+Step 3: Verify that the side menu slides open smoothly.
+Step 4: Check that all 9 categories are listed.</v>
       </c>
       <c r="F12" t="str">
         <v>Mobile drawer opens smoothly and displays all 9 main categories without horizontal scrolling.</v>
@@ -795,10 +795,10 @@
         <v>Mobile menu drawer is open</v>
       </c>
       <c r="E13" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Tap on "Indoor" to expand its subcategories.
-2. Check that child categories expand smoothly.
-3. Tap other categories (Outdoor, Homewares, Support) to expand.
-4. Click subcategory links to test navigation.</v>
+        <v xml:space="preserve">Step 1: Tap on "Indoor" to expand its subcategories.
+Step 2: Check that child categories expand smoothly.
+Step 3: Tap other categories (Outdoor, Homewares, Support) to expand.
+Step 4: Click subcategory links to test navigation.</v>
       </c>
       <c r="F13" t="str">
         <v>Each category accordion expands and collapses cleanly on tap.</v>
@@ -827,10 +827,10 @@
         <v>Desktop view, user on homepage</v>
       </c>
       <c r="E14" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Press Tab key to move focus through the main navigation menu.
-2. Verify visible focus outline around each menu link.
-3. Press Enter or Space to open a dropdown menu.
-4. Use Tab and arrow keys to move through dropdown links.</v>
+        <v xml:space="preserve">Step 1: Press Tab key to move focus through the main navigation menu.
+Step 2: Verify visible focus outline around each menu link.
+Step 3: Press Enter or Space to open a dropdown menu.
+Step 4: Use Tab and arrow keys to move through dropdown links.</v>
       </c>
       <c r="F14" t="str">
         <v>User can navigate all categories and submenu items using keyboard only with clear focus highlighting.</v>
@@ -859,9 +859,9 @@
         <v>A mega menu dropdown is currently open on desktop</v>
       </c>
       <c r="E15" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover or press Enter to open the "Indoor" menu dropdown.
-2. Press the Escape key on your keyboard.
-3. Verify that the dropdown closes immediately.</v>
+        <v xml:space="preserve">Step 1: Hover or press Enter to open the "Indoor" menu dropdown.
+Step 2: Press the Escape key on your keyboard.
+Step 3: Verify that the dropdown closes immediately.</v>
       </c>
       <c r="F15" t="str">
         <v>The dropdown menu should close right away and focus should return to the parent category button.</v>
@@ -890,9 +890,9 @@
         <v>Desktop view, user hovers over main menu</v>
       </c>
       <c r="E16" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover mouse over "Indoor" to open the dropdown.
-2. Move the mouse pointer diagonally towards subcategories on the right.
-3. Verify the menu stays open and does not flicker or close accidentally.</v>
+        <v xml:space="preserve">Step 1: Hover mouse over "Indoor" to open the dropdown.
+Step 2: Move the mouse pointer diagonally towards subcategories on the right.
+Step 3: Verify the menu stays open and does not flicker or close accidentally.</v>
       </c>
       <c r="F16" t="str">
         <v>Dropdown stays open smoothly while moving the mouse pointer across menu columns.</v>
@@ -921,9 +921,9 @@
         <v>User has navigated to a category page like /indoor</v>
       </c>
       <c r="E17" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Click on "Indoor" in the menu to load the Indoor page.
-2. Look at the top navigation bar.
-3. Check if "Indoor" is visually highlighted or underlined to show current page.</v>
+        <v xml:space="preserve">Step 1: Click on "Indoor" in the menu to load the Indoor page.
+Step 2: Look at the top navigation bar.
+Step 3: Check if "Indoor" is visually highlighted or underlined to show current page.</v>
       </c>
       <c r="F17" t="str">
         <v>The current category should show an active underline or bold text so users know where they are.</v>
@@ -952,9 +952,9 @@
         <v>Mega menu dropdown is open on desktop</v>
       </c>
       <c r="E18" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover over any category so the dropdown is open.
-2. Click the Search (magnifying glass) icon in the header.
-3. Check that the mega menu closes automatically and search box opens.</v>
+        <v xml:space="preserve">Step 1: Hover over any category so the dropdown is open.
+Step 2: Click the Search (magnifying glass) icon in the header.
+Step 3: Check that the mega menu closes automatically and search box opens.</v>
       </c>
       <c r="F18" t="str">
         <v>Menu should close cleanly so it does not overlap with the search box.</v>
@@ -983,9 +983,9 @@
         <v>Mobile menu drawer is open on mobile screen</v>
       </c>
       <c r="E19" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. On mobile view, tap hamburger icon to open the side menu.
-2. Tap anywhere on the dimmed background area outside the menu.
-3. Verify that the drawer closes and returns to the page.</v>
+        <v xml:space="preserve">Step 1: On mobile view, tap hamburger icon to open the side menu.
+Step 2: Tap anywhere on the dimmed background area outside the menu.
+Step 3: Verify that the drawer closes and returns to the page.</v>
       </c>
       <c r="F19" t="str">
         <v>Tapping the background overlay should close the menu and re-enable page scrolling.</v>
@@ -1014,9 +1014,9 @@
         <v>Mobile view on mobile phone or emulator</v>
       </c>
       <c r="E20" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open mobile menu drawer.
-2. Tap through several category links.
-3. Check if links have enough spacing so adjacent links are not accidentally tapped.</v>
+        <v xml:space="preserve">Step 1: Open mobile menu drawer.
+Step 2: Tap through several category links.
+Step 3: Check if links have enough spacing so adjacent links are not accidentally tapped.</v>
       </c>
       <c r="F20" t="str">
         <v>Links should have ample height and spacing for easy finger tapping on touchscreens.</v>
@@ -1045,9 +1045,9 @@
         <v>Main menu dropdown is open on desktop</v>
       </c>
       <c r="E21" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Hover over a menu item to open the dropdown.
-2. Click the GlobeWest brand logo in the header.
-3. Verify the browser navigates back to the homepage.</v>
+        <v xml:space="preserve">Step 1: Hover over a menu item to open the dropdown.
+Step 2: Click the GlobeWest brand logo in the header.
+Step 3: Verify the browser navigates back to the homepage.</v>
       </c>
       <c r="F21" t="str">
         <v>Clicking the logo takes the user directly back to the US homepage and closes the menu.</v>
@@ -1076,9 +1076,9 @@
         <v>Storefront loaded with screen reader enabled</v>
       </c>
       <c r="E22" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Focus on category menu items with screen reader on.
-2. Open and close a category dropdown.
-3. Check if the screen reader announces whether the menu is expanded or collapsed.</v>
+        <v xml:space="preserve">Step 1: Focus on category menu items with screen reader on.
+Step 2: Open and close a category dropdown.
+Step 3: Check if the screen reader announces whether the menu is expanded or collapsed.</v>
       </c>
       <c r="F22" t="str">
         <v>Screen reader should announce the category name and state (expanded or collapsed).</v>
@@ -1093,9 +1093,229 @@
         <v>P1 - High</v>
       </c>
     </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC-MM-22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Desktop - Editorial &amp; Promo Cards</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify Promotional Card Display &amp; US Image/Link Parity in Flyouts</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Desktop viewport 1440x900 on US staging homepage</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Hover mouse over categories containing promotional cards (Indoor, Outdoor, Homewares, In Stock).
+Step 2: Inspect right-hand promotional card imagery, heading copy, and CTA button.
+Step 3: Click promotional card CTA and assert target destination URL on US storefront.</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Promotional cards display high-resolution imagery and headlines matching design spec; CTA links navigate cleanly to US collection pages without AU domain leakage.</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Right-hand promotional cards render high-res lifestyle imagery; CTAs link cleanly to US collections with zero Australian domain leakage.</v>
+      </c>
+      <c r="H23" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I23" t="str">
+        <v>P2 - Medium</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC-MM-23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Tablet - Responsive Navigation (768px - 1024px)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify Mega Menu Responsive Breakpoint &amp; Touch Drawer on Tablet / iPad</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Tablet viewport 820x1180 (iPad Air) and 768x1024 (iPad Mini)</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Open US staging homepage on tablet viewport.
+Step 2: Verify header navigation collapses cleanly into mobile hamburger icon at tablet widths.
+Step 3: Tap hamburger icon to open side drawer.
+Step 4: Tap category accordions (Indoor, Outdoor, Support) and test touch interaction.</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Header navigation adapts responsively without horizontal overflow or overlapping logo; side drawer opens smoothly with responsive touch targets.</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Navigation adapts cleanly to tablet viewport; hamburger drawer operates smoothly with comfortable touch spacing across all categories.</v>
+      </c>
+      <c r="H24" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I24" t="str">
+        <v>P1 - High</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC-MM-24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Desktop - Sticky Header on Scroll</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify Mega Menu Flyout Behavior when Header is Sticky on Page Scroll</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Desktop viewport 1440x900, user is on a long PLP or PDP page</v>
+      </c>
+      <c r="E25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Scroll down page past 300px so sticky header locks to top of viewport.
+Step 2: Hover mouse over navigation categories (Indoor, Outdoor, Inspiration).
+Step 3: Verify mega menu flyout dropdown positions correctly below sticky header without clipping or visual lag.</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Mega menu flyout opens directly underneath the sticky header bar with proper z-index layering over page content.</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Mega menu flyout opens seamlessly beneath sticky header; z-index layering sits cleanly above PLP product cards and banners.</v>
+      </c>
+      <c r="H25" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I25" t="str">
+        <v>P2 - Medium</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC-MM-25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Desktop - Primary Category Landing</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify Direct Click on Top-Level Category Navigates to Primary Category PLP</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Desktop viewport 1440x900 on homepage</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Click directly on top-level category label "Indoor" (not subcategory link).
+Step 2: Verify browser navigates to /indoor collection page.
+Step 3: Repeat direct click test for "Outdoor" and "Homewares".</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Direct click on parent category label routes user to the primary category PLP (/indoor, /outdoor, /homewares) with full product catalog.</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Direct clicks route cleanly to respective parent category PLPs on US storefront (/indoor, /outdoor, /homewares) with HTTP 200.</v>
+      </c>
+      <c r="H26" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I26" t="str">
+        <v>P2 - Medium</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>TC-MM-26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Cross-Feature Coexistence - Mini Cart</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Verify Open Mega Menu Flyout Dismisses when Mini Cart Drawer is Opened</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Desktop viewport 1440x900, active open mega menu flyout</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Hover over "Indoor" to expand mega menu flyout.
+Step 2: Click the Mini Cart bag icon in the header.
+Step 3: Verify mega menu flyout automatically closes as mini cart slide-out drawer opens.</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Mega menu flyout closes immediately to avoid visual z-index collision with the cart drawer.</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Mega menu collapses cleanly as mini cart drawer opens; zero z-index or visual overlap conflict.</v>
+      </c>
+      <c r="H27" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I27" t="str">
+        <v>P1 - High</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>TC-MM-27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Dual-Auth Matrix - Trade Customer Session</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Verify Mega Menu Structure and Category Parity in Authenticated Trade Session</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Logged in as approved US Trade customer (deepali.londhe@overdose.digital)</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Log in as Trade customer on US staging.
+Step 2: Inspect top navigation menu bar and all 9 categories.
+Step 3: Hover through Indoor, Outdoor, and In Stock flyouts.
+Step 4: Verify trade pricing toggle and account dropdown coexist alongside mega menu.</v>
+      </c>
+      <c r="F28" t="str">
+        <v>All 9 categories retain full parity with guest view; trade pricing indicator and account utilities render cleanly without displacing category pills.</v>
+      </c>
+      <c r="G28" t="str">
+        <v>All 9 categories render with exact parity in Trade session; header utilities and trade toggle coexist without layout distortion.</v>
+      </c>
+      <c r="H28" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I28" t="str">
+        <v>P1 - High</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>TC-MM-28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Catalog Routing Integrity - Subcategory PLPs</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Verify Core Subcategory Links Navigate to Active US PLP Pages (Zero 404s)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Desktop viewport 1440x900 on US staging</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Hover over "Indoor" and click "Sofas", "Dining Tables", "Lounge Chairs".
+Step 2: Hover over "Outdoor" and click "Dining Tables", "Sofas".
+Step 3: Hover over "In Stock" and click "In Stock Indoor".
+Step 4: Verify all destination pages return HTTP 200 with populated product listing grids.</v>
+      </c>
+      <c r="F29" t="str">
+        <v>All sampled subcategory links route to valid US PLP paths with active product listings and zero 404 error pages.</v>
+      </c>
+      <c r="G29" t="str">
+        <v>All core subcategory links return HTTP 200 with populated product grids and zero 404 broken page errors.</v>
+      </c>
+      <c r="H29" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I29" t="str">
+        <v>P1 - High</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(qa): remove all viewport size and pixel dimension references from Mega Menu test cases
</commit_message>
<xml_diff>
--- a/Sprint-3/MASTER_BACKUP_SPRINT_3/09_Mega_Menu/Mega_Menu_Test_Cases.xlsx
+++ b/Sprint-3/MASTER_BACKUP_SPRINT_3/09_Mega_Menu/Mega_Menu_Test_Cases.xlsx
@@ -760,7 +760,7 @@
         <v>Verify Mobile Menu Drawer Opens and Shows All 9 Categories</v>
       </c>
       <c r="D12" t="str">
-        <v>Mobile view (390x844 on mobile device)</v>
+        <v>User is on mobile browser</v>
       </c>
       <c r="E12" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Open the website on mobile browser.
@@ -1104,7 +1104,7 @@
         <v>Verify Promotional Card Display &amp; US Image/Link Parity in Flyouts</v>
       </c>
       <c r="D23" t="str">
-        <v>Desktop viewport 1440x900 on US staging homepage</v>
+        <v>User is on desktop browser</v>
       </c>
       <c r="E23" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Hover mouse over categories containing promotional cards (Indoor, Outdoor, Homewares, In Stock).
@@ -1129,17 +1129,17 @@
         <v>TC-MM-23</v>
       </c>
       <c r="B24" t="str">
-        <v>Tablet - Responsive Navigation (768px - 1024px)</v>
+        <v>Tablet - Responsive Navigation</v>
       </c>
       <c r="C24" t="str">
         <v>Verify Mega Menu Responsive Breakpoint &amp; Touch Drawer on Tablet / iPad</v>
       </c>
       <c r="D24" t="str">
-        <v>Tablet viewport 820x1180 (iPad Air) and 768x1024 (iPad Mini)</v>
+        <v>User is on tablet browser or device</v>
       </c>
       <c r="E24" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Open US staging homepage on tablet viewport.
-Step 2: Verify header navigation collapses cleanly into mobile hamburger icon at tablet widths.
+Step 2: Verify header navigation collapses cleanly into mobile hamburger icon on tablet view.
 Step 3: Tap hamburger icon to open side drawer.
 Step 4: Tap category accordions (Indoor, Outdoor, Support) and test touch interaction.</v>
       </c>
@@ -1167,10 +1167,10 @@
         <v>Verify Mega Menu Flyout Behavior when Header is Sticky on Page Scroll</v>
       </c>
       <c r="D25" t="str">
-        <v>Desktop viewport 1440x900, user is on a long PLP or PDP page</v>
+        <v>Desktop view, user is on a long page</v>
       </c>
       <c r="E25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Scroll down page past 300px so sticky header locks to top of viewport.
+        <v xml:space="preserve">Step 1: Scroll down the page until the sticky header locks to the top of the screen.
 Step 2: Hover mouse over navigation categories (Indoor, Outdoor, Inspiration).
 Step 3: Verify mega menu flyout dropdown positions correctly below sticky header without clipping or visual lag.</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>Verify Direct Click on Top-Level Category Navigates to Primary Category PLP</v>
       </c>
       <c r="D26" t="str">
-        <v>Desktop viewport 1440x900 on homepage</v>
+        <v>User is on desktop homepage</v>
       </c>
       <c r="E26" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Click directly on top-level category label "Indoor" (not subcategory link).
@@ -1229,7 +1229,7 @@
         <v>Verify Open Mega Menu Flyout Dismisses when Mini Cart Drawer is Opened</v>
       </c>
       <c r="D27" t="str">
-        <v>Desktop viewport 1440x900, active open mega menu flyout</v>
+        <v>Mega menu dropdown is currently open on desktop</v>
       </c>
       <c r="E27" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Hover over "Indoor" to expand mega menu flyout.
@@ -1292,7 +1292,7 @@
         <v>Verify Core Subcategory Links Navigate to Active US PLP Pages (Zero 404s)</v>
       </c>
       <c r="D29" t="str">
-        <v>Desktop viewport 1440x900 on US staging</v>
+        <v>User is on desktop browser</v>
       </c>
       <c r="E29" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Hover over "Indoor" and click "Sofas", "Dining Tables", "Lounge Chairs".

</xml_diff>